<commit_message>
Add typedef value checker traversal
</commit_message>
<xml_diff>
--- a/test/res/typedef.xlsx
+++ b/test/res/typedef.xlsx
@@ -1652,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="14.875" customWidth="1"/>
@@ -1691,8 +1691,10 @@
       <c r="F2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>55</v>
+      <c r="G2" t="inlineStr" s="3">
+        <is>
+          <t>value_checker</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
@@ -2279,8 +2281,10 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="15">
-        <v>71001</v>
+      <c r="A6" t="inlineStr" s="15">
+        <is>
+          <t>71001</t>
+        </is>
       </c>
       <c r="B6" s="16" t="s">
         <v>40</v>

</xml_diff>